<commit_message>
Fixed upload button and note hovering
</commit_message>
<xml_diff>
--- a/MathTutor/questions/question.xlsx
+++ b/MathTutor/questions/question.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\acer\Desktop\zen\maths-tutor-v2\MathTutor\questions\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\zendelona\maths-tutor-v2\MathTutor\questions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFA9DA88-2CC8-430C-9FF7-A68A0F1B0461}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C37A96E-694A-4DCD-AAA8-BB34EA36F18C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="118">
   <si>
     <t>question</t>
   </si>
@@ -159,6 +159,9 @@
     <t>a1:10*b1:10*</t>
   </si>
   <si>
+    <t>{a}*+b}</t>
+  </si>
+  <si>
     <t>{a} % of {b} =</t>
   </si>
   <si>
@@ -229,13 +232,161 @@
   </si>
   <si>
     <t>{a}%{b}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Neha had {a} balloons. She bought {b} more. How many balloons does she have now?
+</t>
+  </si>
+  <si>
+    <t>Tina has {a} crayons. She found {b} more under the table. How many crayons does she have now?</t>
+  </si>
+  <si>
+    <t>A box has {a} chocolates. {b} fell out. How many chocolates remain in the box?</t>
+  </si>
+  <si>
+    <t>a8:12*b1:8*</t>
+  </si>
+  <si>
+    <t>a1:9*b1:4*</t>
+  </si>
+  <si>
+    <t>There are {a} ducks in the pond. {b} more ducks joined. How many ducks are there now?</t>
+  </si>
+  <si>
+    <t>a1:7*b1:10*</t>
+  </si>
+  <si>
+    <t>Meena had {a} pencils. She gave {b} to her friend and bought {c} more. How many pencils does she have now?</t>
+  </si>
+  <si>
+    <t>{a}-{b}+{c}</t>
+  </si>
+  <si>
+    <t>a10:20*b3:8*c5:10*</t>
+  </si>
+  <si>
+    <t>Ramu earns {a} rupees/day. He worked for {b} days and spent {c} rupees. How much is left?</t>
+  </si>
+  <si>
+    <t>a20:50*b3:7*c50:150*</t>
+  </si>
+  <si>
+    <t>{a}×{b}-{c}</t>
+  </si>
+  <si>
+    <t>A movie started at {a} o'clock and ended at {b} o'clock. How long was it?</t>
+  </si>
+  <si>
+    <t>a1:5*b6:10*</t>
+  </si>
+  <si>
+    <t>{b} - {a}</t>
+  </si>
+  <si>
+    <t>An exam started at {a} o'clock and lasted for {b} hours and {c} minutes. How long was the exam?</t>
+  </si>
+  <si>
+    <t>a8:10*b1:2*c15:45*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{b}  + {c} </t>
+  </si>
+  <si>
+    <t>A man works from {a} to {b}, with a break of {c} minutes. How many hours worked?</t>
+  </si>
+  <si>
+    <t>a9:10*b5:6*c30:60*</t>
+  </si>
+  <si>
+    <t>{b}-{a} - {c}/60</t>
+  </si>
+  <si>
+    <t>A plane took off at {a}:{b} and landed at {c}:{d} the next day. What was the flight duration?</t>
+  </si>
+  <si>
+    <t>a11:12*b15:59*c6:8*d15:59*</t>
+  </si>
+  <si>
+    <t>24 - ({a}:{b}) + {c}:{d}30</t>
+  </si>
+  <si>
+    <t>Rahul bought {a} pens at {b} rupees each and {c} books at {d} each. What is the total cost?</t>
+  </si>
+  <si>
+    <t>a2:4*b10:15*c1:3*d20:30*</t>
+  </si>
+  <si>
+    <t>{a}×{b} + {c}×{d}</t>
+  </si>
+  <si>
+    <t>You want to buy items costing {a}, {b}, {c}. You have {d}. Enough money? How much more or less?</t>
+  </si>
+  <si>
+    <t>a30:40*b20:30*c10:20*d80:120*</t>
+  </si>
+  <si>
+    <t>You bought {a} shirts at {b} each and got {c}% discount. What’s the discounted total?</t>
+  </si>
+  <si>
+    <t>a2:4*b500:1000*c10:30*</t>
+  </si>
+  <si>
+    <t>You spent {a}% of {b} on groceries and {c}% on rent. How much money remains?</t>
+  </si>
+  <si>
+    <t>a30:50*b5000:10000*c30:50*</t>
+  </si>
+  <si>
+    <t>{d} - ({a} + {b} + {c})25</t>
+  </si>
+  <si>
+    <t>{a}×{b} - (({a}×{b})×{c}/100)30</t>
+  </si>
+  <si>
+    <t>{b} - ({a}×{b}/100) - ({c}×{b}/100)</t>
+  </si>
+  <si>
+    <t>A bus trip takes {a} hrs and {b} min. Convert total to minutes.</t>
+  </si>
+  <si>
+    <t>{a} × 60 + {b}</t>
+  </si>
+  <si>
+    <t>a1:3* b10:59*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A conference session lasts {a} hrs, {b} min, and {c} sec. Find total seconds. </t>
+  </si>
+  <si>
+    <t>a4,5*b10:59*c15:59*</t>
+  </si>
+  <si>
+    <t>{a}×3600 + {b}×60 + {c} * 40</t>
+  </si>
+  <si>
+    <t>A long trip lasts {a} days, {b} hrs, {c} min, and {d} sec. Convert total to seconds.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> a1,2*b10,11,12*c30:59*d15:59 *</t>
+  </si>
+  <si>
+    <t>{a}×86400 + {b}×3600 + {c}×60 + {d} * 50</t>
+  </si>
+  <si>
+    <t>A train ride lasts {a} hrs and {b} min. Convert total to minutes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a7,8*b45:59* </t>
+  </si>
+  <si>
+    <t>{a} × 60 + {b} * 26</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -249,6 +400,13 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -271,10 +429,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -305,39 +466,39 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0E2841"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="156082"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="E97132"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196B24"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="A02B93"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4EA72E"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="467886"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="96607D"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -389,7 +550,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -500,6 +661,13 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
@@ -508,13 +676,6 @@
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -579,31 +740,11 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -611,13 +752,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="107.21875" customWidth="1"/>
     <col min="2" max="2" width="13.109375" customWidth="1"/>
     <col min="3" max="3" width="42.88671875" customWidth="1"/>
-    <col min="5" max="5" width="14.5546875" customWidth="1"/>
+    <col min="5" max="5" width="30" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
@@ -742,13 +883,13 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>19</v>
+        <v>70</v>
       </c>
       <c r="B7" t="s">
         <v>20</v>
       </c>
       <c r="C7" t="s">
-        <v>21</v>
+        <v>43</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -761,40 +902,40 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
-        <v>23</v>
+      <c r="A8" t="s">
+        <v>74</v>
       </c>
       <c r="B8" t="s">
         <v>20</v>
       </c>
       <c r="C8" t="s">
-        <v>24</v>
+        <v>75</v>
       </c>
       <c r="D8">
         <v>1</v>
       </c>
       <c r="E8" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F8">
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
-        <v>25</v>
+    <row r="9" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
+        <v>69</v>
       </c>
       <c r="B9" t="s">
         <v>20</v>
       </c>
       <c r="C9" t="s">
-        <v>26</v>
+        <v>73</v>
       </c>
       <c r="D9">
         <v>1</v>
       </c>
       <c r="E9" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="F9">
         <v>10</v>
@@ -802,19 +943,19 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="B10" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="C10" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="D10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E10" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F10">
         <v>10</v>
@@ -822,219 +963,219 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>31</v>
+        <v>71</v>
       </c>
       <c r="B11" t="s">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="C11" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="D11">
         <v>1</v>
       </c>
       <c r="E11" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="F11">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>34</v>
+      <c r="A12" s="1" t="s">
+        <v>23</v>
       </c>
       <c r="B12" t="s">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="C12" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12" t="s">
+        <v>17</v>
+      </c>
+      <c r="F12">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13" t="s">
+        <v>26</v>
+      </c>
+      <c r="D13">
+        <v>1</v>
+      </c>
+      <c r="E13" t="s">
+        <v>27</v>
+      </c>
+      <c r="F13">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C14" t="s">
+        <v>78</v>
+      </c>
+      <c r="D14">
         <v>2</v>
       </c>
-      <c r="E12" t="s">
-        <v>22</v>
-      </c>
-      <c r="F12">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>36</v>
-      </c>
-      <c r="B13" t="s">
-        <v>32</v>
-      </c>
-      <c r="C13" t="s">
-        <v>37</v>
-      </c>
-      <c r="D13">
+      <c r="E14" t="s">
+        <v>77</v>
+      </c>
+      <c r="F14">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C15" t="s">
+        <v>80</v>
+      </c>
+      <c r="D15">
         <v>3</v>
       </c>
-      <c r="E13" t="s">
-        <v>17</v>
-      </c>
-      <c r="F13">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>39</v>
-      </c>
-      <c r="B14" t="s">
-        <v>40</v>
-      </c>
-      <c r="C14" t="s">
-        <v>41</v>
-      </c>
-      <c r="D14">
-        <v>1</v>
-      </c>
-      <c r="E14" t="s">
-        <v>38</v>
-      </c>
-      <c r="F14">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>42</v>
-      </c>
-      <c r="B15" t="s">
-        <v>5</v>
-      </c>
-      <c r="C15" t="s">
-        <v>43</v>
-      </c>
-      <c r="D15">
-        <v>1</v>
-      </c>
       <c r="E15" t="s">
-        <v>22</v>
+        <v>81</v>
       </c>
       <c r="F15">
-        <v>5</v>
+        <v>20</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>44</v>
+        <v>28</v>
       </c>
       <c r="B16" t="s">
-        <v>45</v>
+        <v>29</v>
       </c>
       <c r="C16" t="s">
-        <v>46</v>
+        <v>30</v>
       </c>
       <c r="D16">
         <v>2</v>
       </c>
       <c r="E16" t="s">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="F16">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>44</v>
+      <c r="A17" s="1" t="s">
+        <v>94</v>
       </c>
       <c r="B17" t="s">
-        <v>45</v>
+        <v>29</v>
       </c>
       <c r="C17" t="s">
-        <v>48</v>
+        <v>95</v>
       </c>
       <c r="D17">
         <v>3</v>
       </c>
       <c r="E17" t="s">
-        <v>47</v>
+        <v>96</v>
       </c>
       <c r="F17">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>39</v>
+      <c r="A18" s="1" t="s">
+        <v>97</v>
       </c>
       <c r="B18" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="C18" t="s">
-        <v>49</v>
+        <v>98</v>
       </c>
       <c r="D18">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E18" t="s">
-        <v>38</v>
+        <v>103</v>
       </c>
       <c r="F18">
-        <v>10</v>
+        <v>25</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>39</v>
+      <c r="A19" s="1" t="s">
+        <v>99</v>
       </c>
       <c r="B19" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="C19" t="s">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="D19">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E19" t="s">
-        <v>38</v>
+        <v>104</v>
       </c>
       <c r="F19">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>51</v>
+      <c r="A20" s="1" t="s">
+        <v>101</v>
       </c>
       <c r="B20" t="s">
-        <v>52</v>
+        <v>29</v>
       </c>
       <c r="C20" t="s">
-        <v>53</v>
+        <v>102</v>
       </c>
       <c r="D20">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E20" t="s">
-        <v>54</v>
+        <v>105</v>
       </c>
       <c r="F20">
-        <v>5</v>
+        <v>30</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>51</v>
+        <v>31</v>
       </c>
       <c r="B21" t="s">
-        <v>52</v>
+        <v>32</v>
       </c>
       <c r="C21" t="s">
-        <v>55</v>
+        <v>33</v>
       </c>
       <c r="D21">
         <v>1</v>
       </c>
       <c r="E21" t="s">
-        <v>56</v>
+        <v>22</v>
       </c>
       <c r="F21">
         <v>5</v>
@@ -1042,106 +1183,463 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>51</v>
+        <v>34</v>
       </c>
       <c r="B22" t="s">
-        <v>52</v>
+        <v>32</v>
       </c>
       <c r="C22" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="D22">
         <v>2</v>
       </c>
       <c r="E22" t="s">
-        <v>56</v>
+        <v>22</v>
       </c>
       <c r="F22">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="B23" t="s">
-        <v>52</v>
+        <v>32</v>
       </c>
       <c r="C23" t="s">
-        <v>58</v>
+        <v>37</v>
       </c>
       <c r="D23">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E23" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
       <c r="F23">
-        <v>7</v>
+        <v>15</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="2" t="s">
-        <v>59</v>
+      <c r="A24" t="s">
+        <v>39</v>
       </c>
       <c r="B24" t="s">
-        <v>5</v>
+        <v>40</v>
       </c>
       <c r="C24" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="D24">
         <v>1</v>
       </c>
       <c r="E24" t="s">
-        <v>61</v>
+        <v>38</v>
       </c>
       <c r="F24">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>62</v>
+        <v>106</v>
       </c>
       <c r="B25" t="s">
-        <v>40</v>
+        <v>5</v>
       </c>
       <c r="C25" t="s">
-        <v>63</v>
+        <v>108</v>
       </c>
       <c r="D25">
         <v>2</v>
       </c>
       <c r="E25" t="s">
-        <v>64</v>
+        <v>107</v>
       </c>
       <c r="F25">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
+        <v>109</v>
+      </c>
+      <c r="B26" t="s">
+        <v>5</v>
+      </c>
+      <c r="C26" t="s">
+        <v>110</v>
+      </c>
+      <c r="D26">
+        <v>4</v>
+      </c>
+      <c r="E26" t="s">
+        <v>111</v>
+      </c>
+      <c r="F26">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>112</v>
+      </c>
+      <c r="B27" t="s">
+        <v>5</v>
+      </c>
+      <c r="C27" t="s">
+        <v>113</v>
+      </c>
+      <c r="D27">
+        <v>5</v>
+      </c>
+      <c r="E27" t="s">
+        <v>114</v>
+      </c>
+      <c r="F27">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>115</v>
+      </c>
+      <c r="B28" t="s">
+        <v>5</v>
+      </c>
+      <c r="C28" t="s">
+        <v>116</v>
+      </c>
+      <c r="D28">
+        <v>3</v>
+      </c>
+      <c r="E28" t="s">
+        <v>117</v>
+      </c>
+      <c r="F28">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>42</v>
+      </c>
+      <c r="B29" t="s">
+        <v>5</v>
+      </c>
+      <c r="C29" t="s">
+        <v>43</v>
+      </c>
+      <c r="D29">
+        <v>1</v>
+      </c>
+      <c r="E29" t="s">
+        <v>44</v>
+      </c>
+      <c r="F29">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>45</v>
+      </c>
+      <c r="B30" t="s">
+        <v>46</v>
+      </c>
+      <c r="C30" t="s">
+        <v>47</v>
+      </c>
+      <c r="D30">
+        <v>2</v>
+      </c>
+      <c r="E30" t="s">
+        <v>48</v>
+      </c>
+      <c r="F30">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>45</v>
+      </c>
+      <c r="B31" t="s">
+        <v>46</v>
+      </c>
+      <c r="C31" t="s">
+        <v>49</v>
+      </c>
+      <c r="D31">
+        <v>3</v>
+      </c>
+      <c r="E31" t="s">
+        <v>48</v>
+      </c>
+      <c r="F31">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>39</v>
+      </c>
+      <c r="B32" t="s">
+        <v>40</v>
+      </c>
+      <c r="C32" t="s">
+        <v>50</v>
+      </c>
+      <c r="D32">
+        <v>2</v>
+      </c>
+      <c r="E32" t="s">
+        <v>38</v>
+      </c>
+      <c r="F32">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>39</v>
+      </c>
+      <c r="B33" t="s">
+        <v>40</v>
+      </c>
+      <c r="C33" t="s">
+        <v>51</v>
+      </c>
+      <c r="D33">
+        <v>3</v>
+      </c>
+      <c r="E33" t="s">
+        <v>38</v>
+      </c>
+      <c r="F33">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>52</v>
+      </c>
+      <c r="B34" t="s">
+        <v>53</v>
+      </c>
+      <c r="C34" t="s">
+        <v>54</v>
+      </c>
+      <c r="D34">
+        <v>1</v>
+      </c>
+      <c r="E34" t="s">
+        <v>55</v>
+      </c>
+      <c r="F34">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>52</v>
+      </c>
+      <c r="B35" t="s">
+        <v>53</v>
+      </c>
+      <c r="C35" t="s">
+        <v>56</v>
+      </c>
+      <c r="D35">
+        <v>1</v>
+      </c>
+      <c r="E35" t="s">
+        <v>57</v>
+      </c>
+      <c r="F35">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>52</v>
+      </c>
+      <c r="B36" t="s">
+        <v>53</v>
+      </c>
+      <c r="C36" t="s">
+        <v>58</v>
+      </c>
+      <c r="D36">
+        <v>2</v>
+      </c>
+      <c r="E36" t="s">
+        <v>57</v>
+      </c>
+      <c r="F36">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>52</v>
+      </c>
+      <c r="B37" t="s">
+        <v>53</v>
+      </c>
+      <c r="C37" t="s">
+        <v>59</v>
+      </c>
+      <c r="D37">
+        <v>2</v>
+      </c>
+      <c r="E37" t="s">
+        <v>57</v>
+      </c>
+      <c r="F37">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>91</v>
+      </c>
+      <c r="B38" t="s">
+        <v>5</v>
+      </c>
+      <c r="C38" t="s">
+        <v>92</v>
+      </c>
+      <c r="D38">
+        <v>5</v>
+      </c>
+      <c r="E38" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>88</v>
+      </c>
+      <c r="B39" t="s">
+        <v>5</v>
+      </c>
+      <c r="C39" t="s">
+        <v>89</v>
+      </c>
+      <c r="D39">
+        <v>4</v>
+      </c>
+      <c r="E39" t="s">
+        <v>90</v>
+      </c>
+      <c r="F39">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>85</v>
+      </c>
+      <c r="B40" t="s">
+        <v>5</v>
+      </c>
+      <c r="C40" t="s">
+        <v>86</v>
+      </c>
+      <c r="D40">
+        <v>3</v>
+      </c>
+      <c r="E40" t="s">
+        <v>87</v>
+      </c>
+      <c r="F40">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>82</v>
+      </c>
+      <c r="B41" t="s">
+        <v>5</v>
+      </c>
+      <c r="C41" t="s">
+        <v>83</v>
+      </c>
+      <c r="D41">
+        <v>2</v>
+      </c>
+      <c r="E41" t="s">
+        <v>84</v>
+      </c>
+      <c r="F41">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A42" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B42" t="s">
+        <v>5</v>
+      </c>
+      <c r="C42" t="s">
+        <v>61</v>
+      </c>
+      <c r="D42">
+        <v>1</v>
+      </c>
+      <c r="E42" t="s">
+        <v>62</v>
+      </c>
+      <c r="F42">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>63</v>
+      </c>
+      <c r="B43" t="s">
+        <v>40</v>
+      </c>
+      <c r="C43" t="s">
+        <v>64</v>
+      </c>
+      <c r="D43">
+        <v>2</v>
+      </c>
+      <c r="E43" t="s">
         <v>65</v>
       </c>
-      <c r="B26" t="s">
+      <c r="F43">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
         <v>66</v>
       </c>
-      <c r="C26" t="s">
+      <c r="B44" t="s">
+        <v>67</v>
+      </c>
+      <c r="C44" t="s">
         <v>43</v>
       </c>
-      <c r="D26">
-        <v>1</v>
-      </c>
-      <c r="E26" t="s">
-        <v>67</v>
-      </c>
-      <c r="F26">
+      <c r="D44">
+        <v>1</v>
+      </c>
+      <c r="E44" t="s">
+        <v>68</v>
+      </c>
+      <c r="F44">
         <v>10</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>
-  <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
sovled the problems from excel
</commit_message>
<xml_diff>
--- a/MathTutor/questions/question.xlsx
+++ b/MathTutor/questions/question.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\acer\Desktop\zen\maths-tutor-v2\MathTutor\questions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BF48E91-4F17-4412-AC81-61B9E77D5555}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67D54532-F32A-4EA4-9D67-F5DFE9D359EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="117">
   <si>
     <t>question</t>
   </si>
@@ -157,9 +157,6 @@
   </si>
   <si>
     <t>a1:10*b1:10*</t>
-  </si>
-  <si>
-    <t>{a}*+b}</t>
   </si>
   <si>
     <t>{a} % of {b} =</t>
@@ -883,7 +880,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B7" t="s">
         <v>20</v>
@@ -903,13 +900,13 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B8" t="s">
         <v>20</v>
       </c>
       <c r="C8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D8">
         <v>1</v>
@@ -923,13 +920,13 @@
     </row>
     <row r="9" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B9" t="s">
         <v>20</v>
       </c>
       <c r="C9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -963,13 +960,13 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B11" t="s">
         <v>20</v>
       </c>
       <c r="C11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D11">
         <v>1</v>
@@ -1023,19 +1020,19 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B14" t="s">
         <v>20</v>
       </c>
       <c r="C14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D14">
         <v>2</v>
       </c>
       <c r="E14" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F14">
         <v>15</v>
@@ -1043,19 +1040,19 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B15" t="s">
         <v>20</v>
       </c>
       <c r="C15" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D15">
         <v>3</v>
       </c>
       <c r="E15" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F15">
         <v>20</v>
@@ -1083,19 +1080,19 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B17" t="s">
         <v>29</v>
       </c>
       <c r="C17" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D17">
         <v>3</v>
       </c>
       <c r="E17" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F17">
         <v>20</v>
@@ -1103,19 +1100,19 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B18" t="s">
         <v>29</v>
       </c>
       <c r="C18" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D18">
         <v>4</v>
       </c>
       <c r="E18" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F18">
         <v>25</v>
@@ -1123,19 +1120,19 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B19" t="s">
         <v>29</v>
       </c>
       <c r="C19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D19">
         <v>5</v>
       </c>
       <c r="E19" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F19">
         <v>30</v>
@@ -1143,19 +1140,19 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B20" t="s">
         <v>29</v>
       </c>
       <c r="C20" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D20">
         <v>5</v>
       </c>
       <c r="E20" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F20">
         <v>30</v>
@@ -1215,7 +1212,7 @@
         <v>3</v>
       </c>
       <c r="E23" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="F23">
         <v>15</v>
@@ -1243,19 +1240,19 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B25" t="s">
         <v>5</v>
       </c>
       <c r="C25" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D25">
         <v>2</v>
       </c>
       <c r="E25" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F25">
         <v>15</v>
@@ -1263,19 +1260,19 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
+        <v>108</v>
+      </c>
+      <c r="B26" t="s">
+        <v>5</v>
+      </c>
+      <c r="C26" t="s">
         <v>109</v>
-      </c>
-      <c r="B26" t="s">
-        <v>5</v>
-      </c>
-      <c r="C26" t="s">
-        <v>110</v>
       </c>
       <c r="D26">
         <v>4</v>
       </c>
       <c r="E26" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F26">
         <v>30</v>
@@ -1283,19 +1280,19 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
+        <v>111</v>
+      </c>
+      <c r="B27" t="s">
+        <v>5</v>
+      </c>
+      <c r="C27" t="s">
         <v>112</v>
       </c>
-      <c r="B27" t="s">
-        <v>5</v>
-      </c>
-      <c r="C27" t="s">
+      <c r="D27">
+        <v>5</v>
+      </c>
+      <c r="E27" t="s">
         <v>113</v>
-      </c>
-      <c r="D27">
-        <v>5</v>
-      </c>
-      <c r="E27" t="s">
-        <v>114</v>
       </c>
       <c r="F27">
         <v>50</v>
@@ -1303,19 +1300,19 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
+        <v>114</v>
+      </c>
+      <c r="B28" t="s">
+        <v>5</v>
+      </c>
+      <c r="C28" t="s">
         <v>115</v>
-      </c>
-      <c r="B28" t="s">
-        <v>5</v>
-      </c>
-      <c r="C28" t="s">
-        <v>116</v>
       </c>
       <c r="D28">
         <v>3</v>
       </c>
       <c r="E28" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F28">
         <v>25</v>
@@ -1335,7 +1332,7 @@
         <v>1</v>
       </c>
       <c r="E29" t="s">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="F29">
         <v>5</v>
@@ -1343,19 +1340,19 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
+        <v>44</v>
+      </c>
+      <c r="B30" t="s">
         <v>45</v>
       </c>
-      <c r="B30" t="s">
+      <c r="C30" t="s">
         <v>46</v>
-      </c>
-      <c r="C30" t="s">
-        <v>47</v>
       </c>
       <c r="D30">
         <v>2</v>
       </c>
       <c r="E30" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F30">
         <v>5</v>
@@ -1363,19 +1360,19 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
+        <v>44</v>
+      </c>
+      <c r="B31" t="s">
         <v>45</v>
       </c>
-      <c r="B31" t="s">
-        <v>46</v>
-      </c>
       <c r="C31" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D31">
         <v>3</v>
       </c>
       <c r="E31" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F31">
         <v>10</v>
@@ -1389,7 +1386,7 @@
         <v>40</v>
       </c>
       <c r="C32" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D32">
         <v>2</v>
@@ -1409,7 +1406,7 @@
         <v>40</v>
       </c>
       <c r="C33" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D33">
         <v>3</v>
@@ -1423,19 +1420,19 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
+        <v>51</v>
+      </c>
+      <c r="B34" t="s">
         <v>52</v>
       </c>
-      <c r="B34" t="s">
+      <c r="C34" t="s">
         <v>53</v>
       </c>
-      <c r="C34" t="s">
+      <c r="D34">
+        <v>1</v>
+      </c>
+      <c r="E34" t="s">
         <v>54</v>
-      </c>
-      <c r="D34">
-        <v>1</v>
-      </c>
-      <c r="E34" t="s">
-        <v>55</v>
       </c>
       <c r="F34">
         <v>5</v>
@@ -1443,19 +1440,19 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
+        <v>51</v>
+      </c>
+      <c r="B35" t="s">
         <v>52</v>
       </c>
-      <c r="B35" t="s">
-        <v>53</v>
-      </c>
       <c r="C35" t="s">
+        <v>55</v>
+      </c>
+      <c r="D35">
+        <v>1</v>
+      </c>
+      <c r="E35" t="s">
         <v>56</v>
-      </c>
-      <c r="D35">
-        <v>1</v>
-      </c>
-      <c r="E35" t="s">
-        <v>57</v>
       </c>
       <c r="F35">
         <v>5</v>
@@ -1463,19 +1460,19 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
+        <v>51</v>
+      </c>
+      <c r="B36" t="s">
         <v>52</v>
       </c>
-      <c r="B36" t="s">
-        <v>53</v>
-      </c>
       <c r="C36" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D36">
         <v>2</v>
       </c>
       <c r="E36" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F36">
         <v>7</v>
@@ -1483,19 +1480,19 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
+        <v>51</v>
+      </c>
+      <c r="B37" t="s">
         <v>52</v>
       </c>
-      <c r="B37" t="s">
-        <v>53</v>
-      </c>
       <c r="C37" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D37">
         <v>2</v>
       </c>
       <c r="E37" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F37">
         <v>7</v>
@@ -1503,36 +1500,36 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
+        <v>90</v>
+      </c>
+      <c r="B38" t="s">
+        <v>5</v>
+      </c>
+      <c r="C38" t="s">
         <v>91</v>
       </c>
-      <c r="B38" t="s">
-        <v>5</v>
-      </c>
-      <c r="C38" t="s">
+      <c r="D38">
+        <v>5</v>
+      </c>
+      <c r="E38" t="s">
         <v>92</v>
-      </c>
-      <c r="D38">
-        <v>5</v>
-      </c>
-      <c r="E38" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
+        <v>87</v>
+      </c>
+      <c r="B39" t="s">
+        <v>5</v>
+      </c>
+      <c r="C39" t="s">
         <v>88</v>
-      </c>
-      <c r="B39" t="s">
-        <v>5</v>
-      </c>
-      <c r="C39" t="s">
-        <v>89</v>
       </c>
       <c r="D39">
         <v>4</v>
       </c>
       <c r="E39" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F39">
         <v>20</v>
@@ -1540,19 +1537,19 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
+        <v>84</v>
+      </c>
+      <c r="B40" t="s">
+        <v>5</v>
+      </c>
+      <c r="C40" t="s">
         <v>85</v>
-      </c>
-      <c r="B40" t="s">
-        <v>5</v>
-      </c>
-      <c r="C40" t="s">
-        <v>86</v>
       </c>
       <c r="D40">
         <v>3</v>
       </c>
       <c r="E40" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F40">
         <v>15</v>
@@ -1560,19 +1557,19 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
+        <v>81</v>
+      </c>
+      <c r="B41" t="s">
+        <v>5</v>
+      </c>
+      <c r="C41" t="s">
         <v>82</v>
-      </c>
-      <c r="B41" t="s">
-        <v>5</v>
-      </c>
-      <c r="C41" t="s">
-        <v>83</v>
       </c>
       <c r="D41">
         <v>2</v>
       </c>
       <c r="E41" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F41">
         <v>10</v>
@@ -1580,19 +1577,19 @@
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B42" t="s">
+        <v>5</v>
+      </c>
+      <c r="C42" t="s">
         <v>60</v>
       </c>
-      <c r="B42" t="s">
-        <v>5</v>
-      </c>
-      <c r="C42" t="s">
+      <c r="D42">
+        <v>1</v>
+      </c>
+      <c r="E42" t="s">
         <v>61</v>
-      </c>
-      <c r="D42">
-        <v>1</v>
-      </c>
-      <c r="E42" t="s">
-        <v>62</v>
       </c>
       <c r="F42">
         <v>7</v>
@@ -1600,19 +1597,19 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B43" t="s">
         <v>40</v>
       </c>
       <c r="C43" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D43">
         <v>2</v>
       </c>
       <c r="E43" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F43">
         <v>10</v>
@@ -1620,10 +1617,10 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
+        <v>65</v>
+      </c>
+      <c r="B44" t="s">
         <v>66</v>
-      </c>
-      <c r="B44" t="s">
-        <v>67</v>
       </c>
       <c r="C44" t="s">
         <v>43</v>
@@ -1632,7 +1629,7 @@
         <v>1</v>
       </c>
       <c r="E44" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F44">
         <v>10</v>

</xml_diff>